<commit_message>
add script for dataverse
</commit_message>
<xml_diff>
--- a/output/summary_WB_regions_quality_mean_only.xlsx
+++ b/output/summary_WB_regions_quality_mean_only.xlsx
@@ -1733,7 +1733,7 @@
         </is>
       </c>
       <c r="F50">
-        <v>198.6052689339755</v>
+        <v>198.4147578321731</v>
       </c>
     </row>
     <row r="51">
@@ -1758,7 +1758,7 @@
         </is>
       </c>
       <c r="F51">
-        <v>222.2547489332221</v>
+        <v>221.8260445142896</v>
       </c>
     </row>
     <row r="52">
@@ -1783,7 +1783,7 @@
         </is>
       </c>
       <c r="F52">
-        <v>224.9519005721748</v>
+        <v>224.9337516464444</v>
       </c>
     </row>
     <row r="53">
@@ -1808,7 +1808,7 @@
         </is>
       </c>
       <c r="F53">
-        <v>230.4356321178711</v>
+        <v>230.1741136826712</v>
       </c>
     </row>
     <row r="54">
@@ -1833,7 +1833,7 @@
         </is>
       </c>
       <c r="F54">
-        <v>229.4041266420748</v>
+        <v>229.3846627839536</v>
       </c>
     </row>
     <row r="55">
@@ -1883,7 +1883,7 @@
         </is>
       </c>
       <c r="F56">
-        <v>138.1793153409385</v>
+        <v>138.7890091962096</v>
       </c>
     </row>
     <row r="57">
@@ -1908,7 +1908,7 @@
         </is>
       </c>
       <c r="F57">
-        <v>195.6479584136895</v>
+        <v>194.3608927603723</v>
       </c>
     </row>
     <row r="58">
@@ -1938,7 +1938,7 @@
         </is>
       </c>
       <c r="F58">
-        <v>213.6030932611299</v>
+        <v>213.1958780234546</v>
       </c>
     </row>
     <row r="59">
@@ -1968,7 +1968,7 @@
         </is>
       </c>
       <c r="F59">
-        <v>230.7092125071003</v>
+        <v>230.2595086971783</v>
       </c>
     </row>
     <row r="60">
@@ -1998,7 +1998,7 @@
         </is>
       </c>
       <c r="F60">
-        <v>201.0282311307386</v>
+        <v>201.0120052063976</v>
       </c>
     </row>
     <row r="61">
@@ -2028,7 +2028,7 @@
         </is>
       </c>
       <c r="F61">
-        <v>250.385363405146</v>
+        <v>250.3651701197706</v>
       </c>
     </row>
     <row r="62">
@@ -2058,7 +2058,7 @@
         </is>
       </c>
       <c r="F62">
-        <v>214.1853723386369</v>
+        <v>213.9340093386497</v>
       </c>
     </row>
     <row r="63">
@@ -2088,7 +2088,7 @@
         </is>
       </c>
       <c r="F63">
-        <v>247.1386578693536</v>
+        <v>246.8667010474335</v>
       </c>
     </row>
     <row r="64">
@@ -2118,7 +2118,7 @@
         </is>
       </c>
       <c r="F64">
-        <v>206.0105794645407</v>
+        <v>206.0081595397197</v>
       </c>
     </row>
     <row r="65">
@@ -2148,7 +2148,7 @@
         </is>
       </c>
       <c r="F65">
-        <v>251.0343074821435</v>
+        <v>250.9990844338183</v>
       </c>
     </row>
     <row r="66">
@@ -2238,7 +2238,7 @@
         </is>
       </c>
       <c r="F68">
-        <v>130.3323933768629</v>
+        <v>130.9176177733322</v>
       </c>
     </row>
     <row r="69">
@@ -2268,7 +2268,7 @@
         </is>
       </c>
       <c r="F69">
-        <v>145.6472013959224</v>
+        <v>146.2801827428997</v>
       </c>
     </row>
     <row r="70">
@@ -2298,7 +2298,7 @@
         </is>
       </c>
       <c r="F70">
-        <v>177.5906856566514</v>
+        <v>176.4305397891598</v>
       </c>
     </row>
     <row r="71">
@@ -2328,7 +2328,7 @@
         </is>
       </c>
       <c r="F71">
-        <v>213.8645231704046</v>
+        <v>212.4494181100004</v>
       </c>
     </row>
     <row r="72">
@@ -2353,7 +2353,7 @@
         </is>
       </c>
       <c r="F72">
-        <v>185.4839201990257</v>
+        <v>185.3098393960044</v>
       </c>
     </row>
     <row r="73">
@@ -2378,7 +2378,7 @@
         </is>
       </c>
       <c r="F73">
-        <v>211.5541986334455</v>
+        <v>211.3474731326388</v>
       </c>
     </row>
     <row r="74">
@@ -2398,7 +2398,7 @@
         </is>
       </c>
       <c r="F74">
-        <v>239.5795043065802</v>
+        <v>239.3690815816242</v>
       </c>
     </row>
     <row r="75">
@@ -2423,7 +2423,7 @@
         </is>
       </c>
       <c r="F75">
-        <v>277.5001470091651</v>
+        <v>276.9776295916038</v>
       </c>
     </row>
     <row r="76">
@@ -2448,7 +2448,7 @@
         </is>
       </c>
       <c r="F76">
-        <v>273.1911041451213</v>
+        <v>273.1706143819874</v>
       </c>
     </row>
     <row r="77">
@@ -2473,7 +2473,7 @@
         </is>
       </c>
       <c r="F77">
-        <v>278.7329514534464</v>
+        <v>278.5014797052831</v>
       </c>
     </row>
     <row r="78">
@@ -2498,7 +2498,7 @@
         </is>
       </c>
       <c r="F78">
-        <v>265.3026111676061</v>
+        <v>265.0785773807465</v>
       </c>
     </row>
     <row r="79">
@@ -2548,7 +2548,7 @@
         </is>
       </c>
       <c r="F80">
-        <v>162.6257066400563</v>
+        <v>163.3368287992505</v>
       </c>
     </row>
     <row r="81">
@@ -2573,7 +2573,7 @@
         </is>
       </c>
       <c r="F81">
-        <v>220.0638959476481</v>
+        <v>218.7374009283901</v>
       </c>
     </row>
     <row r="82">
@@ -2603,7 +2603,7 @@
         </is>
       </c>
       <c r="F82">
-        <v>266.4149295467641</v>
+        <v>265.9182897247678</v>
       </c>
     </row>
     <row r="83">
@@ -2633,7 +2633,7 @@
         </is>
       </c>
       <c r="F83">
-        <v>288.332705631062</v>
+        <v>287.7849004307477</v>
       </c>
     </row>
     <row r="84">
@@ -2663,7 +2663,7 @@
         </is>
       </c>
       <c r="F84">
-        <v>243.6553601063086</v>
+        <v>243.6370413721139</v>
       </c>
     </row>
     <row r="85">
@@ -2693,7 +2693,7 @@
         </is>
       </c>
       <c r="F85">
-        <v>304.5908127096516</v>
+        <v>304.568014906609</v>
       </c>
     </row>
     <row r="86">
@@ -2723,7 +2723,7 @@
         </is>
       </c>
       <c r="F86">
-        <v>259.0578649060102</v>
+        <v>258.8353836172741</v>
       </c>
     </row>
     <row r="87">
@@ -2753,7 +2753,7 @@
         </is>
       </c>
       <c r="F87">
-        <v>298.9562267566762</v>
+        <v>298.7155140562228</v>
       </c>
     </row>
     <row r="88">
@@ -2783,7 +2783,7 @@
         </is>
       </c>
       <c r="F88">
-        <v>237.6679373476579</v>
+        <v>237.4804903442172</v>
       </c>
     </row>
     <row r="89">
@@ -2813,7 +2813,7 @@
         </is>
       </c>
       <c r="F89">
-        <v>290.85422963938</v>
+        <v>290.596366919452</v>
       </c>
     </row>
     <row r="90">
@@ -2903,7 +2903,7 @@
         </is>
       </c>
       <c r="F92">
-        <v>153.427654430497</v>
+        <v>154.1101100305656</v>
       </c>
     </row>
     <row r="93">
@@ -2933,7 +2933,7 @@
         </is>
       </c>
       <c r="F93">
-        <v>171.3794582567097</v>
+        <v>172.1178622721679</v>
       </c>
     </row>
     <row r="94">
@@ -2963,7 +2963,7 @@
         </is>
       </c>
       <c r="F94">
-        <v>199.7652437605324</v>
+        <v>198.575761608398</v>
       </c>
     </row>
     <row r="95">
@@ -2993,7 +2993,7 @@
         </is>
       </c>
       <c r="F95">
-        <v>240.5416124342901</v>
+        <v>239.0768958906612</v>
       </c>
     </row>
     <row r="96">
@@ -3018,7 +3018,7 @@
         </is>
       </c>
       <c r="F96">
-        <v>223.7331727988306</v>
+        <v>223.5421224540177</v>
       </c>
     </row>
     <row r="97">
@@ -3043,7 +3043,7 @@
         </is>
       </c>
       <c r="F97">
-        <v>255.2176095679521</v>
+        <v>254.9880690225915</v>
       </c>
     </row>
     <row r="98">

</xml_diff>